<commit_message>
fix: cargar asistencias de Actividad 4 en 09/09 para Seccion 1 y Seccion 3 en DB y Excels
</commit_message>
<xml_diff>
--- a/asistencias_excel/Asistencia_Ayudantias_CIT3203_CA01_-_Sección_1_UDP.xlsx
+++ b/asistencias_excel/Asistencia_Ayudantias_CIT3203_CA01_-_Sección_1_UDP.xlsx
@@ -552,7 +552,7 @@
         <v>0</v>
       </c>
       <c r="I5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J5" t="str">
         <v>S/C</v>
@@ -594,16 +594,16 @@
         <v>0.2</v>
       </c>
       <c r="W5">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X5">
         <v>4</v>
       </c>
       <c r="Y5" t="str">
-        <v>50%</v>
+        <v>75%</v>
       </c>
       <c r="Z5" t="str">
-        <v>RI</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="6">
@@ -632,7 +632,7 @@
         <v>1</v>
       </c>
       <c r="I6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J6" t="str">
         <v>S/C</v>
@@ -674,13 +674,13 @@
         <v>0.4</v>
       </c>
       <c r="W6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="X6">
         <v>4</v>
       </c>
       <c r="Y6" t="str">
-        <v>25%</v>
+        <v>50%</v>
       </c>
       <c r="Z6" t="str">
         <v>RI</v>
@@ -712,7 +712,7 @@
         <v>1</v>
       </c>
       <c r="I7">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J7" t="str">
         <v>S/C</v>
@@ -754,13 +754,13 @@
         <v>0.4</v>
       </c>
       <c r="W7">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X7">
         <v>4</v>
       </c>
       <c r="Y7" t="str">
-        <v>75%</v>
+        <v>100%</v>
       </c>
       <c r="Z7" t="str">
         <v>OK</v>
@@ -952,7 +952,7 @@
         <v>1</v>
       </c>
       <c r="I10">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J10" t="str">
         <v>S/C</v>
@@ -994,16 +994,16 @@
         <v>0.6</v>
       </c>
       <c r="W10">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X10">
         <v>4</v>
       </c>
       <c r="Y10" t="str">
-        <v>50%</v>
+        <v>75%</v>
       </c>
       <c r="Z10" t="str">
-        <v>RI</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="11">
@@ -1432,7 +1432,7 @@
         <v>1</v>
       </c>
       <c r="I16">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J16" t="str">
         <v>S/C</v>
@@ -1474,16 +1474,16 @@
         <v>0.4</v>
       </c>
       <c r="W16">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X16">
         <v>4</v>
       </c>
       <c r="Y16" t="str">
-        <v>50%</v>
+        <v>75%</v>
       </c>
       <c r="Z16" t="str">
-        <v>RI</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="17">
@@ -1592,7 +1592,7 @@
         <v>0</v>
       </c>
       <c r="I18">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J18" t="str">
         <v>S/C</v>
@@ -1634,16 +1634,16 @@
         <v>0.6</v>
       </c>
       <c r="W18">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X18">
         <v>4</v>
       </c>
       <c r="Y18" t="str">
-        <v>50%</v>
+        <v>75%</v>
       </c>
       <c r="Z18" t="str">
-        <v>RI</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="19">
@@ -1912,7 +1912,7 @@
         <v>1</v>
       </c>
       <c r="I22">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J22" t="str">
         <v>S/C</v>
@@ -1954,13 +1954,13 @@
         <v>0.2</v>
       </c>
       <c r="W22">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X22">
         <v>4</v>
       </c>
       <c r="Y22" t="str">
-        <v>75%</v>
+        <v>100%</v>
       </c>
       <c r="Z22" t="str">
         <v>OK</v>
@@ -2072,7 +2072,7 @@
         <v>1</v>
       </c>
       <c r="I24">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J24" t="str">
         <v>S/C</v>
@@ -2114,13 +2114,13 @@
         <v>0.2</v>
       </c>
       <c r="W24">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X24">
         <v>4</v>
       </c>
       <c r="Y24" t="str">
-        <v>75%</v>
+        <v>100%</v>
       </c>
       <c r="Z24" t="str">
         <v>OK</v>
@@ -2232,7 +2232,7 @@
         <v>0</v>
       </c>
       <c r="I26">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J26" t="str">
         <v>S/C</v>
@@ -2274,16 +2274,16 @@
         <v>0.4</v>
       </c>
       <c r="W26">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X26">
         <v>4</v>
       </c>
       <c r="Y26" t="str">
-        <v>50%</v>
+        <v>75%</v>
       </c>
       <c r="Z26" t="str">
-        <v>RI</v>
+        <v>OK</v>
       </c>
     </row>
     <row r="27">
@@ -2552,7 +2552,7 @@
         <v>0</v>
       </c>
       <c r="I30">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J30" t="str">
         <v>S/C</v>
@@ -2594,13 +2594,13 @@
         <v>0.2</v>
       </c>
       <c r="W30">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="X30">
         <v>4</v>
       </c>
       <c r="Y30" t="str">
-        <v>25%</v>
+        <v>50%</v>
       </c>
       <c r="Z30" t="str">
         <v>RI</v>
@@ -2712,7 +2712,7 @@
         <v>1</v>
       </c>
       <c r="I32">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J32" t="str">
         <v>S/C</v>
@@ -2754,13 +2754,13 @@
         <v>0.4</v>
       </c>
       <c r="W32">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="X32">
         <v>4</v>
       </c>
       <c r="Y32" t="str">
-        <v>25%</v>
+        <v>50%</v>
       </c>
       <c r="Z32" t="str">
         <v>RI</v>
@@ -2792,7 +2792,7 @@
         <v>17</v>
       </c>
       <c r="I33">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="J33" t="str">
         <v>S/C</v>

</xml_diff>